<commit_message>
documents_uploaded: add PrintSphere_OLH_en-US_draft02 (ID 129, uploaded 2026-06-12)
</commit_message>
<xml_diff>
--- a/documents_uploaded.xlsx
+++ b/documents_uploaded.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEA16715-B04B-451D-B158-DBB7C09FDBBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{773AC410-4C55-478E-A63C-D58BDDEC5F15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{1E54C4EF-5A7A-48A8-A140-BC101A3BE96D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1E54C4EF-5A7A-48A8-A140-BC101A3BE96D}"/>
   </bookViews>
   <sheets>
     <sheet name="Documents" sheetId="1" r:id="rId1"/>
@@ -386,15 +386,9 @@
     <t>User Guide</t>
   </si>
   <si>
-    <t>PrintSphere_OLH_en-US_draft01</t>
-  </si>
-  <si>
     <t>PrintSphere</t>
   </si>
   <si>
-    <t>v3</t>
-  </si>
-  <si>
     <t>Printer, Customer</t>
   </si>
   <si>
@@ -414,6 +408,12 @@
   </si>
   <si>
     <t>TXT</t>
+  </si>
+  <si>
+    <t>v3.0</t>
+  </si>
+  <si>
+    <t>PrintSphere_OLH_en-US_draft02</t>
   </si>
 </sst>
 </file>
@@ -3220,13 +3220,13 @@
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
+        <v>123</v>
+      </c>
+      <c r="B95" t="s">
         <v>114</v>
       </c>
-      <c r="B95" t="s">
-        <v>115</v>
-      </c>
       <c r="D95" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="E95" t="s">
         <v>16</v>
@@ -3238,7 +3238,7 @@
         <v>17</v>
       </c>
       <c r="H95" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="I95" s="3" t="s">
         <v>24</v>
@@ -3246,10 +3246,10 @@
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B96" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E96" t="s">
         <v>16</v>
@@ -3258,7 +3258,7 @@
         <v>108</v>
       </c>
       <c r="G96" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H96" t="s">
         <v>18</v>
@@ -3269,7 +3269,7 @@
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
@@ -3283,13 +3283,13 @@
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F99" t="s">
+        <v>119</v>
+      </c>
+      <c r="G99" t="s">
         <v>121</v>
-      </c>
-      <c r="G99" t="s">
-        <v>123</v>
       </c>
       <c r="I99" s="3" t="s">
         <v>24</v>

</xml_diff>